<commit_message>
Record previous firm history on Business Overview
Save Bob Duncan's confirmed Q2 answer in Business Overview B7:
Rettie Financial Services (5 years); previously Simpson & Marwick, then one year in Aberdeen.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -113,7 +113,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -198,6 +198,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4CC"/>
+        <bgColor rgb="00FFF4CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -441,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -652,6 +658,9 @@
     </xf>
     <xf numFmtId="167" fontId="9" fillId="12" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1475,9 +1484,9 @@
           <t>Previous firm / network</t>
         </is>
       </c>
-      <c r="B7" s="49" t="inlineStr">
-        <is>
-          <t>Rettie Financial Services Ltd / Carrington Mortgage UK Ltd (MAB appointed representative)</t>
+      <c r="B7" s="85" t="inlineStr">
+        <is>
+          <t>Rettie Financial Services (5 years); previously Simpson &amp; Marwick, then one year in Aberdeen</t>
         </is>
       </c>
       <c r="C7" s="52" t="n"/>

</xml_diff>

<commit_message>
Record Bonaly Grove business address
Save Bob Duncan's confirmed Q3 answer in Business Overview B8:
88 Bonaly Grove, Edinburgh, EH13 0QB.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1502,9 +1502,9 @@
           <t>Business address</t>
         </is>
       </c>
-      <c r="B8" s="49" t="inlineStr">
-        <is>
-          <t>Edinburgh and East Lothian — meetings by appointment. Correspondence address TBC on incorporation. Robert.Duncan@duncanandcofinancial.co.uk | 07528523216</t>
+      <c r="B8" s="85" t="inlineStr">
+        <is>
+          <t>88 Bonaly Grove, Edinburgh, EH13 0QB</t>
         </is>
       </c>
       <c r="C8" s="52" t="n"/>

</xml_diff>

<commit_message>
Record Rettie FRN 969595; Duncan & Co FCA TBC
Save Bob's clarification that 969595 is Rettie Financial Services'
FCA/FRN, not a Duncan & Co number. Business Overview B9 is TBC with
that note; B7 now includes FRN 969595 on the Rettie line.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1486,7 +1486,7 @@
       </c>
       <c r="B7" s="85" t="inlineStr">
         <is>
-          <t>Rettie Financial Services (5 years); previously Simpson &amp; Marwick, then one year in Aberdeen</t>
+          <t>Rettie Financial Services (5 years, FRN 969595); previously Simpson &amp; Marwick, then one year in Aberdeen</t>
         </is>
       </c>
       <c r="C7" s="52" t="n"/>
@@ -1520,9 +1520,9 @@
           <t>FCA number</t>
         </is>
       </c>
-      <c r="B9" s="49" t="inlineStr">
-        <is>
-          <t>TBC — intending trading style under Rosemount Financial Solutions (IFA) Ltd FRN 535515</t>
+      <c r="B9" s="85" t="inlineStr">
+        <is>
+          <t>TBC — Rettie Financial Services was FRN 969595</t>
         </is>
       </c>
       <c r="C9" s="52" t="n"/>

</xml_diff>

<commit_message>
Record MAB FCA number as TBC / don't know
Save Bob Duncan's Q5 answer that he does not know the MAB FCA number.
Business Overview B10 is now TBC / don't know.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1538,9 +1538,9 @@
           <t>MAB FCA number</t>
         </is>
       </c>
-      <c r="B10" s="49" t="inlineStr">
-        <is>
-          <t>N/A going forward (previous network MAB Limited FRN 455545; MAB Derby 466154)</t>
+      <c r="B10" s="85" t="inlineStr">
+        <is>
+          <t>TBC / don't know</t>
         </is>
       </c>
       <c r="C10" s="52" t="n"/>

</xml_diff>

<commit_message>
Record L&G master agency number as N/A
Save Bob Duncan's Q6 answer that he does not have an L&G master
agency number. Business Overview B11 is now N/A — don't have one.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1556,9 +1556,9 @@
           <t>L&amp;G master agency number</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B11" s="85" t="inlineStr">
+        <is>
+          <t>N/A — don't have one</t>
         </is>
       </c>
       <c r="C11" s="52" t="n"/>

</xml_diff>

<commit_message>
Record MAB agency number as N/A
Save Bob Duncan's Q7 answer that he does not have a MAB agency
number. Business Overview B12 is now N/A — don't have one.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1574,9 +1574,9 @@
           <t>MAB agency number</t>
         </is>
       </c>
-      <c r="B12" s="49" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B12" s="85" t="inlineStr">
+        <is>
+          <t>N/A — don't have one</t>
         </is>
       </c>
       <c r="C12" s="52" t="n"/>

</xml_diff>

<commit_message>
Record pipeline not novated due to issues
Save Bob Duncan's Q8 answer that no pipeline has been novated
and there are pipeline issues. Business Overview B13 is now
No — none novated (pipeline issues). Later fields left unchanged.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1592,9 +1592,9 @@
           <t>Pipeline novated?</t>
         </is>
       </c>
-      <c r="B13" s="49" t="inlineStr">
-        <is>
-          <t>No — no personal client bank to novate</t>
+      <c r="B13" s="85" t="inlineStr">
+        <is>
+          <t>No — none novated (pipeline issues)</t>
         </is>
       </c>
       <c r="C13" s="52" t="n"/>

</xml_diff>

<commit_message>
Record client fee structure on Business Overview
Save Bob Duncan's Q9 fee structure. Business Overview B14 is now
standard purchase and remortgage £195 on application / £300 on
offer, debt consolidation and adverse £495 / £500, and
international £495 / £1,000. Later fields left unchanged.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1604,15 +1604,15 @@
       <c r="G13" s="52" t="n"/>
       <c r="H13" s="53" t="n"/>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Fee structure</t>
         </is>
       </c>
-      <c r="B14" s="49" t="inlineStr">
-        <is>
-          <t>Lender procuration + protection commission; client fees by agreement on complex / international cases</t>
+      <c r="B14" s="85" t="inlineStr">
+        <is>
+          <t>Standard purchase &amp; remortgage: £195 on application, £300 on offer. Debt consolidation / adverse: £495 on application, £500 on offer. International: £495 on application, £1,000 on offer.</t>
         </is>
       </c>
       <c r="C14" s="52" t="n"/>

</xml_diff>

<commit_message>
Record specialist licences as mortgage, protection, bridging, B&C
Save Bob Duncan's Q10 answer. Business Overview B15 is now
Mortgage and protection; bridging; buy-to-let and commercial (B&C).
B&C read as buy-to-let and commercial. Later fields left unchanged.

Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1628,9 +1628,9 @@
           <t>Specialist licences required</t>
         </is>
       </c>
-      <c r="B15" s="49" t="inlineStr">
-        <is>
-          <t>CeMAP / Cert CII (MP). Later-life / equity release TBC with Rosemount</t>
+      <c r="B15" s="85" t="inlineStr">
+        <is>
+          <t>Mortgage and protection; bridging; buy-to-let and commercial (B&amp;C)</t>
         </is>
       </c>
       <c r="C15" s="52" t="n"/>
@@ -1640,6 +1640,8 @@
       <c r="G15" s="52" t="n"/>
       <c r="H15" s="53" t="n"/>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
         <is>
@@ -1905,6 +1907,8 @@
       <c r="G31" s="36" t="n"/>
       <c r="H31" s="36" t="n"/>
     </row>
+    <row r="32"/>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Record Bob Duncan as the first team row.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1640,8 +1640,6 @@
       <c r="G15" s="52" t="n"/>
       <c r="H15" s="53" t="n"/>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
         <is>
@@ -1699,35 +1697,35 @@
       </c>
       <c r="B20" s="49" t="inlineStr">
         <is>
-          <t>Director / Key Individual</t>
-        </is>
-      </c>
-      <c r="C20" s="50" t="inlineStr">
+          <t>Director / Mortgage &amp; Protection Adviser</t>
+        </is>
+      </c>
+      <c r="C20" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D20" s="50" t="inlineStr">
+      <c r="D20" s="49" t="inlineStr">
         <is>
           <t>Self-employed</t>
         </is>
       </c>
-      <c r="E20" s="50" t="inlineStr">
-        <is>
-          <t>Edinburgh / East Lothian</t>
-        </is>
-      </c>
-      <c r="F20" s="50" t="inlineStr">
-        <is>
-          <t>CeMAP / Cert CII (MP)</t>
-        </is>
-      </c>
-      <c r="G20" s="50" t="inlineStr">
-        <is>
-          <t>Self (launch)</t>
-        </is>
-      </c>
-      <c r="H20" s="50" t="inlineStr">
+      <c r="E20" s="49" t="inlineStr">
+        <is>
+          <t>Edinburgh</t>
+        </is>
+      </c>
+      <c r="F20" s="49" t="inlineStr">
+        <is>
+          <t>Mortgage, protection, bridging, BTL &amp; commercial</t>
+        </is>
+      </c>
+      <c r="G20" s="49" t="inlineStr">
+        <is>
+          <t>No (self at launch)</t>
+        </is>
+      </c>
+      <c r="H20" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1907,8 +1905,6 @@
       <c r="G31" s="36" t="n"/>
       <c r="H31" s="36" t="n"/>
     </row>
-    <row r="32"/>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add lead-out commercial split section; keep team as Bob only.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -447,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -662,6 +662,13 @@
     <xf numFmtId="0" fontId="9" fillId="18" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1732,88 +1739,24 @@
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="49" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="B21" s="49" t="inlineStr">
-        <is>
-          <t>Admin / Case Manager (future)</t>
-        </is>
-      </c>
-      <c r="C21" s="50" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D21" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E21" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F21" s="50" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G21" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="H21" s="50" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="A21" s="86" t="n"/>
+      <c r="B21" s="86" t="n"/>
+      <c r="C21" s="86" t="n"/>
+      <c r="D21" s="86" t="n"/>
+      <c r="E21" s="86" t="n"/>
+      <c r="F21" s="86" t="n"/>
+      <c r="G21" s="86" t="n"/>
+      <c r="H21" s="86" t="n"/>
     </row>
     <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="49" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="B22" s="49" t="inlineStr">
-        <is>
-          <t>Adviser — AR transition (future)</t>
-        </is>
-      </c>
-      <c r="C22" s="50" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D22" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E22" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F22" s="50" t="inlineStr">
-        <is>
-          <t>CeMAP TBC</t>
-        </is>
-      </c>
-      <c r="G22" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="H22" s="50" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="A22" s="86" t="n"/>
+      <c r="B22" s="86" t="n"/>
+      <c r="C22" s="86" t="n"/>
+      <c r="D22" s="86" t="n"/>
+      <c r="E22" s="86" t="n"/>
+      <c r="F22" s="86" t="n"/>
+      <c r="G22" s="86" t="n"/>
+      <c r="H22" s="86" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="36" t="n"/>
@@ -1825,35 +1768,51 @@
       <c r="G23" s="36" t="n"/>
       <c r="H23" s="36" t="n"/>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="36" t="n"/>
-      <c r="B24" s="36" t="n"/>
-      <c r="C24" s="36" t="n"/>
-      <c r="D24" s="36" t="n"/>
-      <c r="E24" s="36" t="n"/>
-      <c r="F24" s="36" t="n"/>
-      <c r="G24" s="36" t="n"/>
-      <c r="H24" s="36" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="36" t="n"/>
-      <c r="B25" s="36" t="n"/>
-      <c r="C25" s="36" t="n"/>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="36" t="n"/>
-      <c r="F25" s="36" t="n"/>
-      <c r="G25" s="36" t="n"/>
-      <c r="H25" s="36" t="n"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="36" t="n"/>
-      <c r="B26" s="36" t="n"/>
-      <c r="C26" s="36" t="n"/>
-      <c r="D26" s="36" t="n"/>
-      <c r="E26" s="36" t="n"/>
-      <c r="F26" s="36" t="n"/>
-      <c r="G26" s="36" t="n"/>
-      <c r="H26" s="36" t="n"/>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>Lead-out and commercial split</t>
+        </is>
+      </c>
+      <c r="B24" s="61" t="n"/>
+      <c r="C24" s="61" t="n"/>
+      <c r="D24" s="61" t="n"/>
+      <c r="E24" s="61" t="n"/>
+      <c r="F24" s="61" t="n"/>
+      <c r="G24" s="61" t="n"/>
+      <c r="H24" s="61" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="87" t="inlineStr">
+        <is>
+          <t>Duncan &amp; Co can pass leads out to specialist advisers (bridging, commercial, BTL, overflow or other work the firm does not keep) for an agreed commercial split.</t>
+        </is>
+      </c>
+      <c r="B25" s="76" t="n"/>
+      <c r="C25" s="76" t="n"/>
+      <c r="D25" s="76" t="n"/>
+      <c r="E25" s="76" t="n"/>
+      <c r="F25" s="76" t="n"/>
+      <c r="G25" s="76" t="n"/>
+      <c r="H25" s="76" t="n"/>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="63" t="inlineStr">
+        <is>
+          <t>Split terms</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>TBC — commercial split to be agreed per introducer / specialist (typical referral-out).</t>
+        </is>
+      </c>
+      <c r="C26" s="88" t="n"/>
+      <c r="D26" s="88" t="n"/>
+      <c r="E26" s="88" t="n"/>
+      <c r="F26" s="88" t="n"/>
+      <c r="G26" s="88" t="n"/>
+      <c r="H26" s="88" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="36" t="n"/>
@@ -2233,13 +2192,16 @@
       <c r="F47" s="36" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="18">
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="B14:H14"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B26:H26"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="B13:H13"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="A34:F34"/>

</xml_diff>

<commit_message>
Record 50/50 lead-out split; client stays with Duncan & Co.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1774,13 +1774,13 @@
           <t>Lead-out and commercial split</t>
         </is>
       </c>
-      <c r="B24" s="61" t="n"/>
-      <c r="C24" s="61" t="n"/>
-      <c r="D24" s="61" t="n"/>
-      <c r="E24" s="61" t="n"/>
-      <c r="F24" s="61" t="n"/>
-      <c r="G24" s="61" t="n"/>
-      <c r="H24" s="61" t="n"/>
+      <c r="B24" s="52" t="n"/>
+      <c r="C24" s="52" t="n"/>
+      <c r="D24" s="52" t="n"/>
+      <c r="E24" s="52" t="n"/>
+      <c r="F24" s="52" t="n"/>
+      <c r="G24" s="52" t="n"/>
+      <c r="H24" s="53" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="87" t="inlineStr">
@@ -1788,13 +1788,13 @@
           <t>Duncan &amp; Co can pass leads out to specialist advisers (bridging, commercial, BTL, overflow or other work the firm does not keep) for an agreed commercial split.</t>
         </is>
       </c>
-      <c r="B25" s="76" t="n"/>
-      <c r="C25" s="76" t="n"/>
-      <c r="D25" s="76" t="n"/>
-      <c r="E25" s="76" t="n"/>
-      <c r="F25" s="76" t="n"/>
-      <c r="G25" s="76" t="n"/>
-      <c r="H25" s="76" t="n"/>
+      <c r="B25" s="52" t="n"/>
+      <c r="C25" s="52" t="n"/>
+      <c r="D25" s="52" t="n"/>
+      <c r="E25" s="52" t="n"/>
+      <c r="F25" s="52" t="n"/>
+      <c r="G25" s="52" t="n"/>
+      <c r="H25" s="53" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="63" t="inlineStr">
@@ -1804,15 +1804,15 @@
       </c>
       <c r="B26" s="49" t="inlineStr">
         <is>
-          <t>TBC — commercial split to be agreed per introducer / specialist (typical referral-out).</t>
-        </is>
-      </c>
-      <c r="C26" s="88" t="n"/>
-      <c r="D26" s="88" t="n"/>
-      <c r="E26" s="88" t="n"/>
-      <c r="F26" s="88" t="n"/>
-      <c r="G26" s="88" t="n"/>
-      <c r="H26" s="88" t="n"/>
+          <t>50/50 split. The customer remains a Duncan &amp; Co Financial customer.</t>
+        </is>
+      </c>
+      <c r="C26" s="52" t="n"/>
+      <c r="D26" s="52" t="n"/>
+      <c r="E26" s="52" t="n"/>
+      <c r="F26" s="52" t="n"/>
+      <c r="G26" s="52" t="n"/>
+      <c r="H26" s="53" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="36" t="n"/>

</xml_diff>

<commit_message>
Record DJ Alexander monthly volume as 5-7 leads.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1919,9 +1919,9 @@
           <t>Estate agent</t>
         </is>
       </c>
-      <c r="D36" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
+      <c r="D36" s="49" t="inlineStr">
+        <is>
+          <t>5–7 leads a month</t>
         </is>
       </c>
       <c r="E36" s="51" t="inlineStr">

</xml_diff>

<commit_message>
Record DJ Alexander close rate as 1 in 3.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -447,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -669,6 +669,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="12" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1924,9 +1927,9 @@
           <t>5–7 leads a month</t>
         </is>
       </c>
-      <c r="E36" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
+      <c r="E36" s="89" t="inlineStr">
+        <is>
+          <t>1 in 3 conversion</t>
         </is>
       </c>
       <c r="F36" s="49" t="inlineStr">

</xml_diff>

<commit_message>
Add Thorntons Solicitors lead source (Hannah Fraser, 3-7 leads).
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -447,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -670,6 +670,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="9" fillId="12" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="13" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1941,226 +1944,74 @@
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="49" t="inlineStr">
         <is>
+          <t>Thorntons Solicitors</t>
+        </is>
+      </c>
+      <c r="B37" s="86" t="n"/>
+      <c r="C37" s="49" t="inlineStr">
+        <is>
+          <t>Solicitor</t>
+        </is>
+      </c>
+      <c r="D37" s="49" t="inlineStr">
+        <is>
+          <t>3–7 leads a month</t>
+        </is>
+      </c>
+      <c r="E37" s="90" t="n"/>
+      <c r="F37" s="49" t="inlineStr">
+        <is>
           <t>Hannah Fraser</t>
         </is>
       </c>
-      <c r="B37" s="49" t="inlineStr">
-        <is>
-          <t>Email / phone introduction</t>
-        </is>
-      </c>
-      <c r="C37" s="49" t="inlineStr">
-        <is>
-          <t>Solicitor / property</t>
-        </is>
-      </c>
-      <c r="D37" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E37" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F37" s="49" t="inlineStr">
-        <is>
-          <t>Senior property partner; agreed primary Edinburgh introducer</t>
-        </is>
-      </c>
     </row>
     <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="49" t="inlineStr">
-        <is>
-          <t>Ralph’s Thayer (Ivan Ralph)</t>
-        </is>
-      </c>
-      <c r="B38" s="49" t="inlineStr">
-        <is>
-          <t>Referral partnership outreach</t>
-        </is>
-      </c>
-      <c r="C38" s="49" t="inlineStr">
-        <is>
-          <t>Referral partner</t>
-        </is>
-      </c>
-      <c r="D38" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E38" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F38" s="49" t="inlineStr">
-        <is>
-          <t>Outreach 2 Sep 2026 — not yet live</t>
-        </is>
-      </c>
+      <c r="A38" s="86" t="n"/>
+      <c r="B38" s="86" t="n"/>
+      <c r="C38" s="86" t="n"/>
+      <c r="D38" s="86" t="n"/>
+      <c r="E38" s="90" t="n"/>
+      <c r="F38" s="86" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="49" t="inlineStr">
-        <is>
-          <t>Glasgow letting / estate agency (via DJ Alexander)</t>
-        </is>
-      </c>
-      <c r="B39" s="49" t="inlineStr">
-        <is>
-          <t>IF confirmed — exclusive</t>
-        </is>
-      </c>
-      <c r="C39" s="49" t="inlineStr">
-        <is>
-          <t>Estate / lettings</t>
-        </is>
-      </c>
-      <c r="D39" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E39" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F39" s="49" t="inlineStr">
-        <is>
-          <t>~2,000–3,000 homes/year discussed; NOT confirmed; high risk</t>
-        </is>
-      </c>
+      <c r="A39" s="86" t="n"/>
+      <c r="B39" s="86" t="n"/>
+      <c r="C39" s="86" t="n"/>
+      <c r="D39" s="86" t="n"/>
+      <c r="E39" s="90" t="n"/>
+      <c r="F39" s="86" t="n"/>
     </row>
     <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="49" t="inlineStr">
-        <is>
-          <t>Website / PPC</t>
-        </is>
-      </c>
-      <c r="B40" s="49" t="inlineStr">
-        <is>
-          <t>Web form</t>
-        </is>
-      </c>
-      <c r="C40" s="49" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="D40" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E40" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F40" s="49" t="inlineStr">
-        <is>
-          <t>Contact Business Gateway for build funding (3 Sep 2026)</t>
-        </is>
-      </c>
+      <c r="A40" s="86" t="n"/>
+      <c r="B40" s="86" t="n"/>
+      <c r="C40" s="86" t="n"/>
+      <c r="D40" s="86" t="n"/>
+      <c r="E40" s="90" t="n"/>
+      <c r="F40" s="86" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="49" t="inlineStr">
-        <is>
-          <t>BoE rate-triggered CRM emails</t>
-        </is>
-      </c>
-      <c r="B41" s="49" t="inlineStr">
-        <is>
-          <t>Email campaign (hold / cut / rise)</t>
-        </is>
-      </c>
-      <c r="C41" s="49" t="inlineStr">
-        <is>
-          <t>Own CRM</t>
-        </is>
-      </c>
-      <c r="D41" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E41" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F41" s="49" t="inlineStr">
-        <is>
-          <t>Intelligent Office sequences; drafted 26 Aug 2026</t>
-        </is>
-      </c>
+      <c r="A41" s="86" t="n"/>
+      <c r="B41" s="86" t="n"/>
+      <c r="C41" s="86" t="n"/>
+      <c r="D41" s="86" t="n"/>
+      <c r="E41" s="90" t="n"/>
+      <c r="F41" s="86" t="n"/>
     </row>
     <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="49" t="inlineStr">
-        <is>
-          <t>Accountant introductions</t>
-        </is>
-      </c>
-      <c r="B42" s="49" t="inlineStr">
-        <is>
-          <t>Professional referral</t>
-        </is>
-      </c>
-      <c r="C42" s="49" t="inlineStr">
-        <is>
-          <t>Accountant</t>
-        </is>
-      </c>
-      <c r="D42" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E42" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F42" s="49" t="inlineStr">
-        <is>
-          <t>Via self-employed / complex cases</t>
-        </is>
-      </c>
+      <c r="A42" s="86" t="n"/>
+      <c r="B42" s="86" t="n"/>
+      <c r="C42" s="86" t="n"/>
+      <c r="D42" s="86" t="n"/>
+      <c r="E42" s="90" t="n"/>
+      <c r="F42" s="86" t="n"/>
     </row>
     <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="49" t="inlineStr">
-        <is>
-          <t>International / overseas buyers</t>
-        </is>
-      </c>
-      <c r="B43" s="49" t="inlineStr">
-        <is>
-          <t>Introducer / website</t>
-        </is>
-      </c>
-      <c r="C43" s="49" t="inlineStr">
-        <is>
-          <t>Specialist</t>
-        </is>
-      </c>
-      <c r="D43" s="50" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E43" s="51" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F43" s="49" t="inlineStr">
-        <is>
-          <t>Edinburgh &amp; St Andrews demand; compliance still to agree with Rosemount</t>
-        </is>
-      </c>
+      <c r="A43" s="86" t="n"/>
+      <c r="B43" s="86" t="n"/>
+      <c r="C43" s="86" t="n"/>
+      <c r="D43" s="86" t="n"/>
+      <c r="E43" s="90" t="n"/>
+      <c r="F43" s="86" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="36" t="n"/>

</xml_diff>

<commit_message>
Match Thorntons delivery and conversion to DJ Alexander.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1947,7 +1947,11 @@
           <t>Thorntons Solicitors</t>
         </is>
       </c>
-      <c r="B37" s="86" t="n"/>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Email introduction (Edinburgh &amp; Lothians)</t>
+        </is>
+      </c>
       <c r="C37" s="49" t="inlineStr">
         <is>
           <t>Solicitor</t>
@@ -1958,7 +1962,11 @@
           <t>3–7 leads a month</t>
         </is>
       </c>
-      <c r="E37" s="90" t="n"/>
+      <c r="E37" s="89" t="inlineStr">
+        <is>
+          <t>1 in 3 conversion</t>
+        </is>
+      </c>
       <c r="F37" s="49" t="inlineStr">
         <is>
           <t>Hannah Fraser</t>

</xml_diff>

<commit_message>
Add TBC system referral lead source at 10-20 a week.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1974,10 +1974,22 @@
       </c>
     </row>
     <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="86" t="n"/>
-      <c r="B38" s="86" t="n"/>
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>TBC — system referral process</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>System-related referral process</t>
+        </is>
+      </c>
       <c r="C38" s="86" t="n"/>
-      <c r="D38" s="86" t="n"/>
+      <c r="D38" s="49" t="inlineStr">
+        <is>
+          <t>10–20 leads a week (estimate)</t>
+        </is>
+      </c>
       <c r="E38" s="90" t="n"/>
       <c r="F38" s="86" t="n"/>
     </row>

</xml_diff>

<commit_message>
Record TBC system source as estate agent.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1984,7 +1984,11 @@
           <t>System-related referral process</t>
         </is>
       </c>
-      <c r="C38" s="86" t="n"/>
+      <c r="C38" s="49" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
       <c r="D38" s="49" t="inlineStr">
         <is>
           <t>10–20 leads a week (estimate)</t>

</xml_diff>

<commit_message>
Record TBC system source close rate as 1 in 3.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1994,7 +1994,11 @@
           <t>10–20 leads a week (estimate)</t>
         </is>
       </c>
-      <c r="E38" s="90" t="n"/>
+      <c r="E38" s="89" t="inlineStr">
+        <is>
+          <t>1 in 3 conversion</t>
+        </is>
+      </c>
       <c r="F38" s="86" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">

</xml_diff>

<commit_message>
Record no owner notes on TBC system lead source.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1999,7 +1999,11 @@
           <t>1 in 3 conversion</t>
         </is>
       </c>
-      <c r="F38" s="86" t="n"/>
+      <c r="F38" s="49" t="inlineStr">
+        <is>
+          <t>No notes</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="86" t="n"/>

</xml_diff>

<commit_message>
Use formal name Robert Duncan as plan owner and team name.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -1705,7 +1705,7 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="49" t="inlineStr">
         <is>
-          <t>Robert (Bob) Duncan</t>
+          <t>Robert Duncan</t>
         </is>
       </c>
       <c r="B20" s="49" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B18" s="49" t="inlineStr">
         <is>
-          <t>Robert (Bob) Duncan</t>
+          <t>Robert Duncan</t>
         </is>
       </c>
       <c r="C18" s="52" t="n"/>

</xml_diff>

<commit_message>
Record 0.35% mortgage income and £180k-£250k case size.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -3599,12 +3599,12 @@
       </c>
       <c r="C12" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="D12" s="56" t="inlineStr">
         <is>
-          <t>Overwrite with actual lender mix. Not a Rosemount quote.</t>
+          <t>Robert Duncan: mortgage income is 0.35% of borrowing. Typical loan £180k–£250k.</t>
         </is>
       </c>
       <c r="E12" s="56" t="inlineStr">
@@ -3714,6 +3714,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="60" t="inlineStr">
         <is>
@@ -5550,7 +5551,7 @@
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="77" t="inlineStr">
         <is>
-          <t>Mortgage cash = Financial Plan mortgage written × yellow procuration % (default 0.35%) × (1 − 10% retention). 12-month view applies the 2-month lag, so Jan–Feb 2027 mortgage/protection cash is nil unless you model 2026 completions.</t>
+          <t>Typical completed mortgage: £180,000–£250,000. Income = 0.35% of that borrowing (confirmed by Robert).</t>
         </is>
       </c>
       <c r="B81" s="52" t="n"/>
@@ -5572,7 +5573,7 @@
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="56" t="inlineStr">
         <is>
-          <t>Network fee £75/week = £325/month is Confirmed. 10% mortgage and 15% protection retention are Confirmed (Ahmed Bawa, 2 Sep 2026).</t>
+          <t>Named sources only (DJ 5–7 + Thorntons 3–7, 1 in 3): about 3–5 completions/month. Mid written ≈ £790k; mid income before network ≈ £2,800.</t>
         </is>
       </c>
       <c r="B82" s="52" t="n"/>
@@ -5594,7 +5595,7 @@
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="77" t="inlineStr">
         <is>
-          <t>Sole trader vs limited company is still open (20 Aug consult). Wife is a teacher ~£25–26k and a possible shareholder — tax advice sits with the accountant, not this sheet.</t>
+          <t>If TBC system 10–20/week is included at 1 in 3, written jumps to several million a month. Decide whether that sits in the 2027 target.</t>
         </is>
       </c>
       <c r="B83" s="52" t="n"/>

</xml_diff>

<commit_message>
Set mortgage written target to £790k from named lead sources.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -447,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -673,6 +673,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="13" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2805,15 +2808,15 @@
           <t>Mortgage</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>1035000</v>
+      <c r="B7" s="91" t="n">
+        <v>790000</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="38" t="inlineStr">
         <is>
-          <t>New Build and Retention combined</t>
+          <t>Named sources only (DJ Alexander + Thorntons). Mid-point of 3–5 completions × £180k–£250k. Income = 0.35% of this written amount.</t>
         </is>
       </c>
       <c r="E7" s="40" t="n"/>
@@ -3714,7 +3717,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="60" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Set protection to £1,000 per case, 1-3 cases a month.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -2828,15 +2828,15 @@
           <t>Protection</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
-        <v>240000</v>
+      <c r="B8" s="91" t="n">
+        <v>2000</v>
       </c>
       <c r="C8" s="36" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="38" t="inlineStr">
         <is>
-          <t>Protection income</t>
+          <t>Cash: £1,000 per protection case; 1–3 cases a month (mid £2,000). Not a large written-volume figure.</t>
         </is>
       </c>
       <c r="E8" s="40" t="n"/>
@@ -3623,16 +3623,16 @@
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="C13" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t>Cash assumption — NOT the £240k protection written figure.</t>
+          <t>Robert: £1,000 per case, 1–3 cases a month. Mid-point £2,000 cash before 15% retention.</t>
         </is>
       </c>
       <c r="E13" s="56" t="inlineStr">

</xml_diff>

<commit_message>
Record confirmed office, laptop, web, AI and setup costs.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -3939,11 +3939,11 @@
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="63" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Office subscription</t>
         </is>
       </c>
       <c r="B26" s="64" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C26" s="50" t="inlineStr">
         <is>
@@ -3952,12 +3952,12 @@
       </c>
       <c r="D26" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E26" s="56" t="inlineStr">
         <is>
-          <t>Business standard / equivalent.</t>
+          <t>Office subscription (Robert).</t>
         </is>
       </c>
       <c r="F26" s="66">
@@ -4026,11 +4026,11 @@
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="63" t="inlineStr">
         <is>
-          <t>Domain / email</t>
+          <t>Domain name and website</t>
         </is>
       </c>
       <c r="B29" s="64" t="n">
-        <v>15</v>
+        <v>14.99</v>
       </c>
       <c r="C29" s="50" t="inlineStr">
         <is>
@@ -4039,12 +4039,12 @@
       </c>
       <c r="D29" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E29" s="56" t="inlineStr">
         <is>
-          <t>duncanandcofinancial.co.uk.</t>
+          <t>Domain name and website together.</t>
         </is>
       </c>
       <c r="F29" s="66">
@@ -4055,11 +4055,11 @@
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="63" t="inlineStr">
         <is>
-          <t>Web hosting</t>
+          <t>Web hosting (included above)</t>
         </is>
       </c>
       <c r="B30" s="64" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C30" s="50" t="inlineStr">
         <is>
@@ -4068,12 +4068,12 @@
       </c>
       <c r="D30" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E30" s="56" t="inlineStr">
         <is>
-          <t>If not bundled with the website grant.</t>
+          <t>Included in the £14.99 domain/website line.</t>
         </is>
       </c>
       <c r="F30" s="66">
@@ -4084,11 +4084,11 @@
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="63" t="inlineStr">
         <is>
-          <t>AI / productivity tools</t>
+          <t>AI package</t>
         </is>
       </c>
       <c r="B31" s="64" t="n">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="C31" s="50" t="inlineStr">
         <is>
@@ -4097,12 +4097,12 @@
       </c>
       <c r="D31" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E31" s="56" t="inlineStr">
         <is>
-          <t>Grok / Cursor / similar.</t>
+          <t>AI package (Robert).</t>
         </is>
       </c>
       <c r="F31" s="66">
@@ -4229,11 +4229,11 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="63" t="inlineStr">
         <is>
-          <t>Stationery / postage</t>
+          <t>Laptop (monthly)</t>
         </is>
       </c>
       <c r="B36" s="64" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C36" s="50" t="inlineStr">
         <is>
@@ -4242,12 +4242,12 @@
       </c>
       <c r="D36" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E36" s="56" t="inlineStr">
         <is>
-          <t>IDV, packs, post.</t>
+          <t>Laptop on a monthly basis (Robert).</t>
         </is>
       </c>
       <c r="F36" s="66">
@@ -4357,7 +4357,7 @@
         </is>
       </c>
       <c r="B42" s="70" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C42" s="50" t="inlineStr">
         <is>
@@ -4366,12 +4366,12 @@
       </c>
       <c r="D42" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Moved</t>
         </is>
       </c>
       <c r="E42" s="56" t="inlineStr">
         <is>
-          <t>Replace / dedicated work machine.</t>
+          <t>Laptop is £50/month in operating costs, not a one-off.</t>
         </is>
       </c>
       <c r="F42" s="56" t="inlineStr">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="B43" s="70" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="C43" s="50" t="inlineStr">
         <is>
@@ -4396,12 +4396,12 @@
       </c>
       <c r="D43" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Included</t>
         </is>
       </c>
       <c r="E43" s="56" t="inlineStr">
         <is>
-          <t>Or Business Gateway funded — set to 0 if grant covers it.</t>
+          <t>Website is in the £14.99 monthly domain/website line.</t>
         </is>
       </c>
       <c r="F43" s="56" t="inlineStr">
@@ -4416,8 +4416,8 @@
           <t>Company formation</t>
         </is>
       </c>
-      <c r="B44" s="70" t="n">
-        <v>50</v>
+      <c r="B44" s="64" t="n">
+        <v>480</v>
       </c>
       <c r="C44" s="50" t="inlineStr">
         <is>
@@ -4426,12 +4426,12 @@
       </c>
       <c r="D44" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E44" s="56" t="inlineStr">
         <is>
-          <t>If limited company route is chosen (20 Aug consult).</t>
+          <t>£400 + VAT for business registration and setup.</t>
         </is>
       </c>
       <c r="F44" s="56" t="inlineStr">

</xml_diff>

<commit_message>
Remove Tesla lease from business costs (personal name).
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -3798,7 +3798,7 @@
         </is>
       </c>
       <c r="B21" s="64" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="C21" s="50" t="inlineStr">
         <is>
@@ -3807,12 +3807,12 @@
       </c>
       <c r="D21" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E21" s="56" t="inlineStr">
         <is>
-          <t>Amount UNKNOWN — 3 years remaining. Transfer needs lessor approval.</t>
+          <t>Tesla Model Y is in Robert’s personal name — not a business cost.</t>
         </is>
       </c>
       <c r="F21" s="66">

</xml_diff>

<commit_message>
Ignore EV insurance and charging on business costs.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="B22" s="64" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="C22" s="50" t="inlineStr">
         <is>
@@ -3836,12 +3836,12 @@
       </c>
       <c r="D22" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Ignored</t>
         </is>
       </c>
       <c r="E22" s="56" t="inlineStr">
         <is>
-          <t>Overwrite with actual schedule.</t>
+          <t>Ignored — not a business cost for this plan.</t>
         </is>
       </c>
       <c r="F22" s="66">
@@ -3856,7 +3856,7 @@
         </is>
       </c>
       <c r="B23" s="64" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="C23" s="50" t="inlineStr">
         <is>
@@ -3865,12 +3865,12 @@
       </c>
       <c r="D23" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Ignored</t>
         </is>
       </c>
       <c r="E23" s="56" t="inlineStr">
         <is>
-          <t>Electricity for the Tesla; will vary.</t>
+          <t>Ignored — not a business cost for this plan.</t>
         </is>
       </c>
       <c r="F23" s="66">

</xml_diff>

<commit_message>
Confirm mobile phone at £45 a month.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -3894,12 +3894,12 @@
       </c>
       <c r="D24" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E24" s="56" t="inlineStr">
         <is>
-          <t>Business mobile.</t>
+          <t>£45/month — confirmed by Robert.</t>
         </is>
       </c>
       <c r="F24" s="66">

</xml_diff>

<commit_message>
Leave broadband share at £30.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -3923,12 +3923,12 @@
       </c>
       <c r="D25" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E25" s="56" t="inlineStr">
         <is>
-          <t>Home-office share.</t>
+          <t>£30 home-office share — left as is by Robert.</t>
         </is>
       </c>
       <c r="F25" s="66">

</xml_diff>

<commit_message>
Confirm accountant accrual at £150 a month.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -4010,12 +4010,12 @@
       </c>
       <c r="D28" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E28" s="56" t="inlineStr">
         <is>
-          <t>Monthly accrual; year-end extra not included.</t>
+          <t>£150/month accrual — confirmed by Robert.</t>
         </is>
       </c>
       <c r="F28" s="66">

</xml_diff>

<commit_message>
Confirm Xero at £33 a month.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -3981,12 +3981,12 @@
       </c>
       <c r="D27" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E27" s="56" t="inlineStr">
         <is>
-          <t>Bookkeeping subscription.</t>
+          <t>£33/month Xero — confirmed by Robert.</t>
         </is>
       </c>
       <c r="F27" s="66">

</xml_diff>

<commit_message>
Set marketing spend to zero.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="B32" s="64" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="C32" s="50" t="inlineStr">
         <is>
@@ -4126,12 +4126,12 @@
       </c>
       <c r="D32" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E32" s="56" t="inlineStr">
         <is>
-          <t>Light brand and lead support.</t>
+          <t>Set to £0 by Robert.</t>
         </is>
       </c>
       <c r="F32" s="66">

</xml_diff>

<commit_message>
Set client gifts to zero.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -4146,7 +4146,7 @@
         </is>
       </c>
       <c r="B33" s="64" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C33" s="50" t="inlineStr">
         <is>
@@ -4155,12 +4155,12 @@
       </c>
       <c r="D33" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E33" s="56" t="inlineStr">
         <is>
-          <t>Keep modest in year 1.</t>
+          <t>Set to £0 by Robert.</t>
         </is>
       </c>
       <c r="F33" s="66">

</xml_diff>

<commit_message>
Confirm business bank fees at £10 a month.
Co-authored-by: boab21mac <boab21mac@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/duncan-and-co-planning/Strategic_planning.xlsx
+++ b/duncan-and-co-planning/Strategic_planning.xlsx
@@ -4184,12 +4184,12 @@
       </c>
       <c r="D34" s="50" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="E34" s="56" t="inlineStr">
         <is>
-          <t>Account fees.</t>
+          <t>£10/month bank fees — confirmed by Robert.</t>
         </is>
       </c>
       <c r="F34" s="66">

</xml_diff>